<commit_message>
Update daily_log_tracker: Day 4 complete (6/7)
- Day 4 block date → 2026-05-27; D4-01–D4-06 marked Done with evidence notes.
- D4-07 manual theme validation: In Progress (190-row sample pending review).
- Day4_Done sheet filled with theme pipeline metrics and file paths.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/google play/docs/daily_logs/daily_log_tracker.xlsx
+++ b/google play/docs/daily_logs/daily_log_tracker.xlsx
@@ -2777,7 +2777,7 @@
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Day 4 - 2026-05-08</t>
+          <t>Day 4 - 2026-05-27</t>
         </is>
       </c>
       <c r="B25" s="8" t="n"/>
@@ -2793,7 +2793,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -2823,21 +2823,29 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I26" s="5" t="inlineStr"/>
-      <c r="J26" s="5" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>themes.yml v2 (18 themes, 13 neg + 5 pos, exclude rules)</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -2867,21 +2875,29 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I27" s="5" t="inlineStr"/>
-      <c r="J27" s="5" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>scripts/06_insights/build_review_themes.py</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>19:32</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -2911,21 +2927,29 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I28" s="5" t="inlineStr"/>
-      <c r="J28" s="5" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>reviews_with_themes.csv (10940 rows; coverage 45.2%)</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>19:32</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -2955,21 +2979,29 @@
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I29" s="5" t="inlineStr"/>
-      <c r="J29" s="5" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>theme_summary_overall/by_app + low_star_theme_summary</t>
+        </is>
+      </c>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>19:33</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
@@ -2999,21 +3031,29 @@
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I30" s="5" t="inlineStr"/>
-      <c r="J30" s="5" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>v1→v2: Fun FP 462→382; Difficulty 29→113; Account→3</t>
+        </is>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -3043,21 +3083,29 @@
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="I31" s="5" t="inlineStr"/>
-      <c r="J31" s="5" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>docs/daily_logs/day4_2026-05-27.md</t>
+        </is>
+      </c>
+      <c r="J31" s="5" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3092,7 +3140,12 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>theme_validation_sample.csv (190 rows); manual Y/N pending Day 5</t>
         </is>
       </c>
     </row>
@@ -5224,6 +5277,11 @@
           <t>Date</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Owner</t>
@@ -5278,13 +5336,21 @@
           <t>themes.yml_created</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>18 themes (13 neg + 5 pos), v2 with exclude rules</t>
+        </is>
+      </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>config/themes.yml</t>
+        </is>
+      </c>
       <c r="F6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
@@ -5298,13 +5364,21 @@
           <t>reviews_with_themes.csv</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>10940 rows, multi-label</t>
+        </is>
+      </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>data/processed/reviews_with_themes.csv</t>
+        </is>
+      </c>
       <c r="F7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
@@ -5318,13 +5392,21 @@
           <t>theme_coverage_rate</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr"/>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>45.2% (≥1 theme)</t>
+        </is>
+      </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>reports/tables/theme_summary_overall.csv</t>
+        </is>
+      </c>
       <c r="F8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
@@ -5338,13 +5420,21 @@
           <t>low_star_theme_topN</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr"/>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Fun 12.2%; Crash 8.1%; Loading 5.7%; Pay-to-win 3.9%; Difficulty 3.6%</t>
+        </is>
+      </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>reports/tables/low_star_theme_summary.csv</t>
+        </is>
+      </c>
       <c r="F9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
@@ -5358,13 +5448,21 @@
           <t>positive_theme_topN</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr"/>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Fun n=3567 share=32.6%; Story n=519; Visual n=239; Social n=230</t>
+        </is>
+      </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>reports/tables/theme_summary_overall.csv</t>
+        </is>
+      </c>
       <c r="F10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
@@ -5378,13 +5476,21 @@
           <t>manual_theme_QA_round1</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr"/>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>v1→v2 calibrated; 190-row sample generated; manual Y/N pending</t>
+        </is>
+      </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>reports/tables/theme_validation_sample.csv</t>
+        </is>
+      </c>
       <c r="F11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
@@ -5398,13 +5504,21 @@
           <t>day_conclusion</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr"/>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Theme pipeline shipped; Crash rating_gap +1.28; Loading +1.08 → Day 5 Priority</t>
+        </is>
+      </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>docs/daily_logs/day4_2026-05-27.md</t>
+        </is>
+      </c>
       <c r="F12" s="5" t="inlineStr"/>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Day 6: mark Tableau dashboard completion in logs/tracker
Close D6-01 to D6-04 as done in Tableau on macOS and align the Day 6 status narrative with the final delivery path.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/google play/docs/daily_logs/daily_log_tracker.xlsx
+++ b/google play/docs/daily_logs/daily_log_tracker.xlsx
@@ -3583,20 +3583,24 @@
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I42" s="5" t="inlineStr">
         <is>
-          <t>Power BI manual build pending; mockup ready at figures/01_top_bottom_health.png + dashboard_build_guide.md §3</t>
-        </is>
-      </c>
-      <c r="J42" s="5" t="n"/>
+          <t>Tableau Page 1 built in Mobile_Game_Satisfaction_Tableau.twbx (Executive Overview).</t>
+        </is>
+      </c>
+      <c r="J42" s="5" t="inlineStr">
+        <is>
+          <t>03:21</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
@@ -3631,20 +3635,24 @@
       </c>
       <c r="G43" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr">
         <is>
-          <t>Power BI manual build pending; mockup ready at figures/02_*.png, 03_*.png + dashboard_build_guide.md §4</t>
-        </is>
-      </c>
-      <c r="J43" s="5" t="n"/>
+          <t>Tableau Page 2 built in Mobile_Game_Satisfaction_Tableau.twbx (Competitor Benchmark).</t>
+        </is>
+      </c>
+      <c r="J43" s="5" t="inlineStr">
+        <is>
+          <t>03:21</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -3679,20 +3687,24 @@
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I44" s="5" t="inlineStr">
         <is>
-          <t>Power BI manual build pending; mockup ready at figures/04..06_*.png + dashboard_build_guide.md §5</t>
-        </is>
-      </c>
-      <c r="J44" s="5" t="n"/>
+          <t>Tableau Page 3 built in Mobile_Game_Satisfaction_Tableau.twbx (Theme Insights).</t>
+        </is>
+      </c>
+      <c r="J44" s="5" t="inlineStr">
+        <is>
+          <t>03:21</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
@@ -3727,20 +3739,24 @@
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr">
         <is>
-          <t>Power BI manual build pending; mockup ready at figures/07..08_*.png + dashboard_build_guide.md §6</t>
-        </is>
-      </c>
-      <c r="J45" s="5" t="n"/>
+          <t>Tableau Page 4 built in Mobile_Game_Satisfaction_Tableau.twbx (Product Recommendation).</t>
+        </is>
+      </c>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t>03:21</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
@@ -6193,20 +6209,24 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Mockup at figures/01_top_bottom_health.png; build guide §3</t>
+          <t>Tableau Page 1 complete (Executive Overview).</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>docs/dashboard_build_guide.md</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr"/>
+          <t>reports/每日复盘/Mobile_Game_Satisfaction_Tableau.twbx</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>dashboard_page1.png captured</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -6221,20 +6241,24 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Mockups at figures/02_*.png, 03_*.png; build guide §4</t>
+          <t>Tableau Page 2 complete (Competitor Benchmark).</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>docs/dashboard_build_guide.md</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr"/>
+          <t>reports/每日复盘/Mobile_Game_Satisfaction_Tableau.twbx</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>dashboard_page2.png captured</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -6249,20 +6273,24 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Mockups at figures/04..06_*.png; build guide §5</t>
+          <t>Tableau Page 3 complete (Theme Insights).</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>docs/dashboard_build_guide.md</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr"/>
+          <t>reports/每日复盘/Mobile_Game_Satisfaction_Tableau.twbx</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>dashboard_page3.png captured</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -6277,20 +6305,24 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Mockups at figures/07..08_*.png; build guide §6</t>
+          <t>Tableau Page 4 complete (Product Recommendation).</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>docs/dashboard_build_guide.md</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr"/>
+          <t>reports/每日复盘/Mobile_Game_Satisfaction_Tableau.twbx</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>dashboard_page4.png captured</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -6361,7 +6393,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Day 6 narrative + figures done; Power BI manual build pending</t>
+          <t>Day 6 dashboard + report deliverables complete; Tableau build finished on macOS.</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -6374,7 +6406,7 @@
           <t>docs/daily_logs/day6_2026-05-28.md</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr"/>
+      <c r="F12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -6390,7 +6422,7 @@
       <c r="C13" s="5" t="n"/>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E13" s="5" t="n"/>

</xml_diff>